<commit_message>
Completed dependency matrix, added the design principles and architectural constraints worksheets
</commit_message>
<xml_diff>
--- a/docs/project-management/03_Design/hld/Northwind-Solution-Capability-Catalogue.xlsx
+++ b/docs/project-management/03_Design/hld/Northwind-Solution-Capability-Catalogue.xlsx
@@ -8,15 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d752cb73b61fc091/Desktop/linuxlabs/projectredstone/docs/project-management/03_Design/hld/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="410" documentId="11_AD4DB114E441178AC67DF4981653DACC693EDF26" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A467F7D7-1C40-4BAA-B2E9-95638BAE26C2}"/>
+  <xr:revisionPtr revIDLastSave="604" documentId="11_AD4DB114E441178AC67DF4981653DACC693EDF26" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{21609EE1-163E-4F03-AD74-A6723E0A05BA}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{73B8EBFB-0F4C-4490-A86A-2BCFFEC2DE0D}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{73B8EBFB-0F4C-4490-A86A-2BCFFEC2DE0D}"/>
   </bookViews>
   <sheets>
     <sheet name="Capabilities" sheetId="1" r:id="rId1"/>
     <sheet name="Dependency Matrix" sheetId="2" r:id="rId2"/>
+    <sheet name="ArchitecturalConstraints" sheetId="3" r:id="rId3"/>
+    <sheet name="Design Principles" sheetId="4" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dependency Matrix'!$A$1:$H$44</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -27,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="753" uniqueCount="312">
   <si>
     <t>Capability ID</t>
   </si>
@@ -329,15 +334,9 @@
     <t>Hard technical</t>
   </si>
   <si>
-    <t>Logging</t>
-  </si>
-  <si>
     <t>Operational</t>
   </si>
   <si>
-    <t>Soft / Design Dependent</t>
-  </si>
-  <si>
     <t>Hard Technical</t>
   </si>
   <si>
@@ -347,15 +346,9 @@
     <t>Dependency Bias (Intrinsic/Requirement-derived/Design-dependent)</t>
   </si>
   <si>
-    <t>Who are you going to alert</t>
-  </si>
-  <si>
     <t>Configuration of planned automations need to be stored somewhere so they can be loaded and run.</t>
   </si>
   <si>
-    <t>Logs of what triggered in the background should be kept so they can be reviewed</t>
-  </si>
-  <si>
     <t>Such operations require computation power / effort</t>
   </si>
   <si>
@@ -363,6 +356,618 @@
   </si>
   <si>
     <t>Admins can configure additional or existing storage volumes when required</t>
+  </si>
+  <si>
+    <t>Intrinsic</t>
+  </si>
+  <si>
+    <t>Requirement-derived</t>
+  </si>
+  <si>
+    <t>Design-dependent</t>
+  </si>
+  <si>
+    <t>Design-dependent &amp; Requirement-derived</t>
+  </si>
+  <si>
+    <t>Design Note</t>
+  </si>
+  <si>
+    <t>IAM will facilitate the ability to alert specific users or groups of users based on their permissions</t>
+  </si>
+  <si>
+    <t>Monitoring and alerting applications may need the ability to interface with other tools, services, hardware to check their current status</t>
+  </si>
+  <si>
+    <t>Compute resources required to run programs checking services</t>
+  </si>
+  <si>
+    <t>Users need a way to connect to their machine remotely, IAM ensures that you can access your own device and files</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remote access attempts should be logged to identify suspicious vs normal activity. </t>
+  </si>
+  <si>
+    <t>Solutions needed to enable admins remote access ability to devices on the network and for users outside the company network to connect to their devices</t>
+  </si>
+  <si>
+    <t>The ability to integrate with other tools, services, software is dependent on network connectivity for transmitting data</t>
+  </si>
+  <si>
+    <t>Service integration requires a level of compute processing</t>
+  </si>
+  <si>
+    <t>Logs should be enabled to track operations performed by integration</t>
+  </si>
+  <si>
+    <t>Logs of what triggered in the background should be kept so they can be reviewed, this provides evidence of execution, outcome and failures.</t>
+  </si>
+  <si>
+    <t>Centralised logs may be fed into tools to generate alerts</t>
+  </si>
+  <si>
+    <t>Measurements need trustworthy timestamps, incident timelines need reconstruction</t>
+  </si>
+  <si>
+    <t>Remote access requires processing resources and execution environments for the services/endpoints that establish and terminate remote sessions.</t>
+  </si>
+  <si>
+    <t>Soft Technical</t>
+  </si>
+  <si>
+    <t>Operational and audit information provides source data required for some Northwind reports and historical analysis.</t>
+  </si>
+  <si>
+    <t>Monitoring provides health, availability, utilisation and performance data required for operational/capacity reporting.</t>
+  </si>
+  <si>
+    <t>Asset information provides inventory, ownership, lifecycle and configuration data required for relevant management reports.</t>
+  </si>
+  <si>
+    <t>Consistent timestamps allow information from different systems and periods to be accurately correlated and reported.</t>
+  </si>
+  <si>
+    <t>Northwind requires software and updates to be obtained and managed across multiple systems; loss of connectivity would constrain centralised distribution and administration.</t>
+  </si>
+  <si>
+    <t>Patch-management processes operate against compute workloads and require suitable environments for testing updates before wider deployment.</t>
+  </si>
+  <si>
+    <t>Authorised administrators must be able to assess, approve, deploy, troubleshoot and, where necessary, reverse software changes.</t>
+  </si>
+  <si>
+    <t>Northwind requires evidence of update activity, outcomes and failures to support troubleshooting and controlled change.</t>
+  </si>
+  <si>
+    <t>Recoverability is required where software changes cause service or system failure and cannot be safely corrected through normal rollback mechanisms.</t>
+  </si>
+  <si>
+    <t>Centralised time synchronisation requires network communication between time sources and participating systems.</t>
+  </si>
+  <si>
+    <t>If Northwind operates its own time service, an execution environment will be required to provide that service. An external/appliance-based design could alter this dependency.</t>
+  </si>
+  <si>
+    <t>Administrators require the ability to configure time sources, validate synchronisation and investigate clock-related problems.</t>
+  </si>
+  <si>
+    <t>Compute resources must be provisioned, configured, maintained and troubleshot throughout their lifecycle.</t>
+  </si>
+  <si>
+    <t>Storage Provisioning / Management</t>
+  </si>
+  <si>
+    <t>Many compute workloads require persistent storage, although the precise dependency depends on the eventual compute/storage architecture.</t>
+  </si>
+  <si>
+    <t>Northwind compute workloads need network connectivity to provide and consume infrastructure and business services, although compute itself can technically operate without network connectivity.</t>
+  </si>
+  <si>
+    <t>Northwind requires administrative access to be attributable to authorised identities and governed by appropriate privileges.</t>
+  </si>
+  <si>
+    <t>Northwind requires administrators to securely manage infrastructure remotely; local administration remains possible during remote-access failure.</t>
+  </si>
+  <si>
+    <t>Administrative actions must be sufficiently recorded to support accountability, troubleshooting and incident investigation.</t>
+  </si>
+  <si>
+    <t>Centralised/remote administration of distributed infrastructure relies on network connectivity, although local management may remain possible.</t>
+  </si>
+  <si>
+    <t>Administrative mechanisms must operate within Northwind's security controls, including privileged-access restrictions and host protections.</t>
+  </si>
+  <si>
+    <t>Security controls rely on trustworthy identity and authorisation information for user- and administrator-specific enforcement.</t>
+  </si>
+  <si>
+    <t>Security investigation and accountability require reliable records of security-relevant system and user activity.</t>
+  </si>
+  <si>
+    <t>Security-relevant conditions must be detectable and capable of generating actionable alerts.</t>
+  </si>
+  <si>
+    <t>Some protective controls operate at network boundaries or between network segments, while host-based controls may continue independently.</t>
+  </si>
+  <si>
+    <t>Timely remediation of known software vulnerabilities is an important part of maintaining system security.</t>
+  </si>
+  <si>
+    <t>Reliable timestamps are required to correlate security events and reconstruct incident timelines.</t>
+  </si>
+  <si>
+    <t>Asset and configuration information must be maintained as infrastructure is introduced, changed and retired.</t>
+  </si>
+  <si>
+    <t>Change history and administrative records support traceability of changes to managed assets and configurations.</t>
+  </si>
+  <si>
+    <t>Structured asset information may be automatically collected, validated or consumed by administrative scripts, but Northwind can initially maintain the register manually.</t>
+  </si>
+  <si>
+    <t>Governance &amp; Approval Workflow Support</t>
+  </si>
+  <si>
+    <t>Where approval workflows are implemented, participants and approvers need to be identifiable and appropriately authorised.</t>
+  </si>
+  <si>
+    <t>Approval decisions and associated actions should be traceable for accountability and later review.</t>
+  </si>
+  <si>
+    <t>Automated approval workflows may need to exchange requests or decisions with other systems, but this depends on how the conditional capability is implemented.</t>
+  </si>
+  <si>
+    <t>Constraint ID</t>
+  </si>
+  <si>
+    <t>Constraint</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Applies To</t>
+  </si>
+  <si>
+    <t>Architectural Effect</t>
+  </si>
+  <si>
+    <t>CON-001</t>
+  </si>
+  <si>
+    <t>Security by Design</t>
+  </si>
+  <si>
+    <t>Security; Data Protection; Host Security Enforcement; Network Security BRs</t>
+  </si>
+  <si>
+    <t>All infrastructure capabilities</t>
+  </si>
+  <si>
+    <t>The architecture must incorporate appropriate security controls throughout the solution rather than relying on a single security layer. Access, communications, administration, hosted services and stored data must be protected according to their risk and business purpose.</t>
+  </si>
+  <si>
+    <t>CON-002</t>
+  </si>
+  <si>
+    <t>Least-Privilege Access</t>
+  </si>
+  <si>
+    <t>Security; Identity &amp; Access BRs; Administrative Approval Workflows</t>
+  </si>
+  <si>
+    <t>IAM, File &amp; Data Services, Remote Access, Systems Administration, Application Hosting, Security</t>
+  </si>
+  <si>
+    <t>Users, services and administrators must receive only the access required to perform approved functions. Architectural designs should support role-based and appropriately scoped privileges rather than unrestricted administrative or user access.</t>
+  </si>
+  <si>
+    <t>CON-003</t>
+  </si>
+  <si>
+    <t>Recoverable Operations</t>
+  </si>
+  <si>
+    <t>Recoverable Operations NFR; Recoverability; Backup &amp; Recovery BRs; Software Update Governance</t>
+  </si>
+  <si>
+    <t>Compute, Storage, File Services, Application Hosting, Patch Management, IAM, Administration</t>
+  </si>
+  <si>
+    <t>The architecture must support recovery from configuration errors, failed changes, software failures and infrastructure incidents. Components that materially affect business services must have an appropriate recovery mechanism.</t>
+  </si>
+  <si>
+    <t>CON-004</t>
+  </si>
+  <si>
+    <t>Proportionate Availability and Resilience</t>
+  </si>
+  <si>
+    <t>Availability; Reliability; Business Service Continuity; Service Recovery; Application Resilience</t>
+  </si>
+  <si>
+    <t>Business-critical services, Compute, Network, Storage, IAM, Application Hosting, File Services</t>
+  </si>
+  <si>
+    <t>Resilience must be proportionate to business impact and agreed recovery objectives. Single points of failure should be identified and consciously accepted, mitigated or removed rather than automatically introducing high-availability technology everywhere.</t>
+  </si>
+  <si>
+    <t>CON-005</t>
+  </si>
+  <si>
+    <t>Operational Consistency and Standardisation</t>
+  </si>
+  <si>
+    <t>Operational Consistency; Maintainability; Infrastructure Standardisation BR</t>
+  </si>
+  <si>
+    <t>Compute, Storage, IAM, Patch Management, Administration, Automation, Hosted Services</t>
+  </si>
+  <si>
+    <t>Infrastructure should use documented, repeatable and consistent configuration and operational patterns wherever practical. Unnecessary variation between systems should be minimised to reduce administrative effort and human error.</t>
+  </si>
+  <si>
+    <t>CON-006</t>
+  </si>
+  <si>
+    <t>Observable and Auditable Operations</t>
+  </si>
+  <si>
+    <t>Monitoring &amp; Observability; Auditability; Centralised Logging; Operational Monitoring BRs</t>
+  </si>
+  <si>
+    <t>All managed infrastructure and services</t>
+  </si>
+  <si>
+    <t>Important services and infrastructure must provide sufficient health, event and activity information to support proactive operations, troubleshooting, auditing and incident investigation. Significant administrative and security-relevant activity should be traceable.</t>
+  </si>
+  <si>
+    <t>CON-007</t>
+  </si>
+  <si>
+    <t>Consistent Time Reference</t>
+  </si>
+  <si>
+    <t>Time Consistency NFR; System Time Consistency BR</t>
+  </si>
+  <si>
+    <t>Logging, Monitoring, IAM, Security, Automation, Network Services, Hosted Applications</t>
+  </si>
+  <si>
+    <t>Supported systems must use a sufficiently consistent time reference to allow reliable authentication, scheduling, event correlation, monitoring and incident investigation.</t>
+  </si>
+  <si>
+    <t>CON-008</t>
+  </si>
+  <si>
+    <t>Controlled and Recoverable Change</t>
+  </si>
+  <si>
+    <t>Software &amp; System Update Management; Software &amp; Package Lifecycle Management; Recoverable Operations; Operational Consistency</t>
+  </si>
+  <si>
+    <t>Patch Management, Compute, Application Hosting, Administration, Automation</t>
+  </si>
+  <si>
+    <t>Infrastructure changes must be performed through controlled and repeatable processes. Where changes present meaningful service risk, the design must allow testing, validation and practical rollback or recovery.</t>
+  </si>
+  <si>
+    <t>CON-009</t>
+  </si>
+  <si>
+    <t>Secure Administrative Access</t>
+  </si>
+  <si>
+    <t>Remote Administration; Secure Remote Access; Security; Auditability</t>
+  </si>
+  <si>
+    <t>Systems Administration, Network, Compute, IAM, Remote Access</t>
+  </si>
+  <si>
+    <t>Administrative mechanisms must authenticate authorised administrators, constrain privileges appropriately and support accountability. Remote administration must not require unnecessary exposure of management interfaces or services.</t>
+  </si>
+  <si>
+    <t>CON-010</t>
+  </si>
+  <si>
+    <t>Interoperability with Existing Services</t>
+  </si>
+  <si>
+    <t>Compatibility; Integration with Existing Business Services BR</t>
+  </si>
+  <si>
+    <t>IAM, Network, Application Hosting, File Services, Reporting, Administration</t>
+  </si>
+  <si>
+    <t>New infrastructure must be capable of interoperating with required existing Northwind services without introducing unnecessary replacement or duplication. Technology choices must consider compatibility with existing business dependencies.</t>
+  </si>
+  <si>
+    <t>CON-011</t>
+  </si>
+  <si>
+    <t>Scalable Without Unnecessary Complexity</t>
+  </si>
+  <si>
+    <t>Scalability; Extensibility; Infrastructure Scalability BR; Administrative Simplicity</t>
+  </si>
+  <si>
+    <t>Compute, Storage, Network, File Services, Application Hosting, Monitoring</t>
+  </si>
+  <si>
+    <t>The architecture must accommodate foreseeable Northwind growth without requiring fundamental redesign, while avoiding complexity introduced purely for hypothetical future scale. Expansion should be achievable through understandable and supportable changes.</t>
+  </si>
+  <si>
+    <t>CON-012</t>
+  </si>
+  <si>
+    <t>Supportable and Maintainable Design</t>
+  </si>
+  <si>
+    <t>Maintainability; Supportability; Administrative Simplicity; Operational Documentation</t>
+  </si>
+  <si>
+    <t>All managed infrastructure</t>
+  </si>
+  <si>
+    <t>The solution must remain understandable and operable by Northwind administrators. Designs requiring excessive specialist knowledge, unnecessary components or undocumented dependencies should be avoided where simpler approaches meet the requirements.</t>
+  </si>
+  <si>
+    <t>CON-013</t>
+  </si>
+  <si>
+    <t>Business Data Segregation and Protection</t>
+  </si>
+  <si>
+    <t>Data Protection; Secure File Services; Departmental Data Segregation; Secure Data Access</t>
+  </si>
+  <si>
+    <t>File &amp; Data Services, Storage, IAM, Backup, Security</t>
+  </si>
+  <si>
+    <t>Business information must be logically protected according to ownership, sensitivity and authorised access. Protection requirements must remain applicable to primary data, backups and recovery operations.</t>
+  </si>
+  <si>
+    <t>CON-014</t>
+  </si>
+  <si>
+    <t>Capacity and Performance Visibility</t>
+  </si>
+  <si>
+    <t>Performance; Capacity &amp; Performance Management; Reporting &amp; Visibility</t>
+  </si>
+  <si>
+    <t>Compute, Storage, Network, Application Hosting, Monitoring, Reporting</t>
+  </si>
+  <si>
+    <t>The architecture must provide sufficient visibility of utilisation and performance to identify emerging constraints and support evidence-based capacity planning before business services are materially affected.</t>
+  </si>
+  <si>
+    <t>Principle ID</t>
+  </si>
+  <si>
+    <t>Design Principle</t>
+  </si>
+  <si>
+    <t>Rationale</t>
+  </si>
+  <si>
+    <t>Design Implication</t>
+  </si>
+  <si>
+    <t>DP-001</t>
+  </si>
+  <si>
+    <t>Requirements-Led Technology Selection</t>
+  </si>
+  <si>
+    <t>Northwind’s infrastructure should exist to satisfy approved business and operational requirements, not to introduce technology for its own sake.</t>
+  </si>
+  <si>
+    <t>Technologies, platforms and architectural patterns should only be introduced where they clearly support an approved requirement, capability, constraint or justified future need.</t>
+  </si>
+  <si>
+    <t>DP-002</t>
+  </si>
+  <si>
+    <t>Prefer Simplicity Over Unnecessary Complexity</t>
+  </si>
+  <si>
+    <t>Simpler systems are generally easier to understand, operate, troubleshoot, secure and recover.</t>
+  </si>
+  <si>
+    <t>Where multiple solutions meet the requirements, preference should be given to the least complex option that remains supportable, secure and sufficiently scalable.</t>
+  </si>
+  <si>
+    <t>DP-003</t>
+  </si>
+  <si>
+    <t>Standardise Where Practical</t>
+  </si>
+  <si>
+    <t>Consistency reduces configuration drift, human error, troubleshooting effort and operational overhead.</t>
+  </si>
+  <si>
+    <t>Common build patterns, configuration approaches, directory structures, administrative procedures and service conventions should be reused across the environment unless a justified exception exists.</t>
+  </si>
+  <si>
+    <t>DP-004</t>
+  </si>
+  <si>
+    <t>Design for Recoverability</t>
+  </si>
+  <si>
+    <t>Northwind requires recovery from operational errors, failed changes and infrastructure incidents.</t>
+  </si>
+  <si>
+    <t>Services and infrastructure should be designed so that important configuration, data and service state can be restored using documented and practical recovery mechanisms.</t>
+  </si>
+  <si>
+    <t>DP-005</t>
+  </si>
+  <si>
+    <t>Apply Proportionate Resilience</t>
+  </si>
+  <si>
+    <t>Not every service requires high availability, but critical services should not contain unexamined failure points.</t>
+  </si>
+  <si>
+    <t>Single points of failure must be identified and assessed against business impact and recovery objectives. Resilience should be added where justified rather than applied universally.</t>
+  </si>
+  <si>
+    <t>DP-006</t>
+  </si>
+  <si>
+    <t>Enforce Least Privilege</t>
+  </si>
+  <si>
+    <t>Excessive access increases both accidental and malicious risk.</t>
+  </si>
+  <si>
+    <t>Users, administrators and services should receive only the permissions required for their approved functions. Administrative access should be separated from ordinary user access where appropriate.</t>
+  </si>
+  <si>
+    <t>DP-007</t>
+  </si>
+  <si>
+    <t>Use Defence in Depth</t>
+  </si>
+  <si>
+    <t>No single control should be assumed to provide complete protection.</t>
+  </si>
+  <si>
+    <t>Security should be applied across identity, hosts, networks, remote access, applications, logging and administrative processes rather than relying on one perimeter control or product.</t>
+  </si>
+  <si>
+    <t>DP-008</t>
+  </si>
+  <si>
+    <t>Make Operations Observable and Auditable</t>
+  </si>
+  <si>
+    <t>Northwind must be able to determine system health, investigate incidents and understand significant changes.</t>
+  </si>
+  <si>
+    <t>Important infrastructure and services should produce useful monitoring, logging and audit information, and those records should use consistent time references where required.</t>
+  </si>
+  <si>
+    <t>DP-009</t>
+  </si>
+  <si>
+    <t>Treat Administrative Access as a Controlled Service</t>
+  </si>
+  <si>
+    <t>Administrative access is one of the highest-risk functions within the infrastructure.</t>
+  </si>
+  <si>
+    <t>Administration should use authorised identities, appropriate privilege boundaries, secure access mechanisms and auditable actions. Management interfaces should not be exposed more broadly than necessary.</t>
+  </si>
+  <si>
+    <t>DP-010</t>
+  </si>
+  <si>
+    <t>Prefer Controlled and Reversible Change</t>
+  </si>
+  <si>
+    <t>Patching and configuration changes can introduce outages or regressions.</t>
+  </si>
+  <si>
+    <t>Changes should be testable, documented and recoverable. Where practical, rollback or restore mechanisms should exist before potentially disruptive changes are implemented.</t>
+  </si>
+  <si>
+    <t>DP-011</t>
+  </si>
+  <si>
+    <t>Separate Responsibilities Where It Improves Control</t>
+  </si>
+  <si>
+    <t>Combining unrelated functions can increase security risk, failure impact and administrative complexity.</t>
+  </si>
+  <si>
+    <t>Capabilities such as identity, administration, monitoring, backup and security should remain logically distinct even where they may share infrastructure or technology.</t>
+  </si>
+  <si>
+    <t>DP-012</t>
+  </si>
+  <si>
+    <t>Avoid Unnecessary Coupling</t>
+  </si>
+  <si>
+    <t>Strong coupling increases failure propagation and can make recovery more difficult.</t>
+  </si>
+  <si>
+    <t>Services should depend only on capabilities genuinely required for their operation. Circular dependencies should be minimised or supported by documented recovery paths.</t>
+  </si>
+  <si>
+    <t>DP-013</t>
+  </si>
+  <si>
+    <t>Design for Managed Growth</t>
+  </si>
+  <si>
+    <t>Northwind expects the environment to expand, but premature enterprise complexity would increase cost and operational burden.</t>
+  </si>
+  <si>
+    <t>The architecture should permit reasonable increases in users, data, systems and workloads without fundamental redesign while avoiding technologies justified only by hypothetical future scale.</t>
+  </si>
+  <si>
+    <t>DP-014</t>
+  </si>
+  <si>
+    <t>Preserve Interoperability</t>
+  </si>
+  <si>
+    <t>New infrastructure must coexist with Northwind’s existing business services.</t>
+  </si>
+  <si>
+    <t>Design choices should use appropriate standards and interfaces and avoid unnecessary dependencies that prevent integration with existing or future systems.</t>
+  </si>
+  <si>
+    <t>DP-015</t>
+  </si>
+  <si>
+    <t>Prefer Automation for Repeatable Operations, Not Understanding Replacement</t>
+  </si>
+  <si>
+    <t>Automation reduces variation and administrative effort, but poorly understood automation can magnify errors.</t>
+  </si>
+  <si>
+    <t>Repetitive and scheduled tasks should be candidates for automation once their manual process, expected outcome, failure modes and recovery method are understood.</t>
+  </si>
+  <si>
+    <t>DP-016</t>
+  </si>
+  <si>
+    <t>Design for Supportability</t>
+  </si>
+  <si>
+    <t>Northwind needs infrastructure that its administrators can understand, maintain and troubleshoot over time.</t>
+  </si>
+  <si>
+    <t>Architectural choices should favour documented, well-understood and maintainable solutions over unnecessarily specialised or opaque implementations.</t>
+  </si>
+  <si>
+    <t>DP-017</t>
+  </si>
+  <si>
+    <t>Protect Business Data Throughout Its Lifecycle</t>
+  </si>
+  <si>
+    <t>Sensitive information remains sensitive whether active, stored, transferred, backed up or restored.</t>
+  </si>
+  <si>
+    <t>Access control, segregation and protection requirements should remain applicable to primary data, backups, recovery operations and administrative access paths.</t>
+  </si>
+  <si>
+    <t>DP-018</t>
+  </si>
+  <si>
+    <t>Time Is a Shared Infrastructure Dependency</t>
+  </si>
+  <si>
+    <t>Authentication, logging, monitoring, automation and investigation all depend on sufficiently consistent timestamps.</t>
+  </si>
+  <si>
+    <t>Infrastructure should use a common and reliable time reference and avoid isolated systems whose clock behaviour could undermine other services.</t>
   </si>
 </sst>
 </file>
@@ -424,7 +1029,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -437,11 +1042,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -450,11 +1050,70 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="6">
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -465,6 +1124,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -987,7 +1650,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5B8861B-C05D-461E-8A99-E228C4472CAF}">
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:L76"/>
   <sheetFormatPr defaultColWidth="27.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
@@ -996,7 +1659,7 @@
     <col min="7" max="7" width="46.42578125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1013,16 +1676,20 @@
         <v>94</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="H1" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="J1" s="5"/>
+      <c r="L1" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1038,14 +1705,18 @@
       <c r="E2" s="2" t="s">
         <v>99</v>
       </c>
+      <c r="F2" s="2" t="s">
+        <v>108</v>
+      </c>
       <c r="G2" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="J2" s="5"/>
+      <c r="L2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -1061,12 +1732,18 @@
       <c r="E3" s="2" t="s">
         <v>99</v>
       </c>
+      <c r="F3" s="2" t="s">
+        <v>108</v>
+      </c>
       <c r="G3" s="2" t="s">
         <v>86</v>
       </c>
       <c r="J3" s="5"/>
-    </row>
-    <row r="4" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="L3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1080,14 +1757,20 @@
         <v>25</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>109</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>80</v>
       </c>
       <c r="J4" s="5"/>
-    </row>
-    <row r="5" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="L4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -1103,12 +1786,18 @@
       <c r="E5" s="2" t="s">
         <v>99</v>
       </c>
+      <c r="F5" s="2" t="s">
+        <v>108</v>
+      </c>
       <c r="G5" s="2" t="s">
         <v>87</v>
       </c>
       <c r="J5" s="5"/>
-    </row>
-    <row r="6" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="L5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -1122,98 +1811,113 @@
         <v>21</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>104</v>
+        <v>99</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>111</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>88</v>
       </c>
       <c r="J6" s="5"/>
     </row>
-    <row r="7" spans="1:10" s="12" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
+    <row r="7" spans="1:12" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="7" t="s">
         <v>13</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E7" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="G7" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="J7" s="9"/>
-    </row>
-    <row r="8" spans="1:10" s="12" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
+      <c r="F7" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="J7" s="6"/>
+    </row>
+    <row r="8" spans="1:12" s="9" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="7" t="s">
         <v>13</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="J8" s="9"/>
-    </row>
-    <row r="9" spans="1:10" s="12" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
+      <c r="E8" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="J8" s="6"/>
+    </row>
+    <row r="9" spans="1:12" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="7" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="E9" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="G9" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="J9" s="9"/>
-    </row>
-    <row r="10" spans="1:10" s="12" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
+      <c r="E9" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="J9" s="6"/>
+    </row>
+    <row r="10" spans="1:12" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="7" t="s">
         <v>13</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="E10" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="G10" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="J10" s="9"/>
-    </row>
-    <row r="11" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="F10" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="J10" s="6"/>
+    </row>
+    <row r="11" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>29</v>
       </c>
@@ -1229,14 +1933,14 @@
       <c r="E11" s="2" t="s">
         <v>99</v>
       </c>
+      <c r="F11" s="2" t="s">
+        <v>108</v>
+      </c>
       <c r="G11" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="J11" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -1252,12 +1956,14 @@
       <c r="E12" s="2" t="s">
         <v>99</v>
       </c>
+      <c r="F12" s="2" t="s">
+        <v>108</v>
+      </c>
       <c r="G12" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="J12" s="5"/>
-    </row>
-    <row r="13" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>29</v>
       </c>
@@ -1273,12 +1979,14 @@
       <c r="E13" s="2" t="s">
         <v>99</v>
       </c>
+      <c r="F13" s="2" t="s">
+        <v>108</v>
+      </c>
       <c r="G13" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="J13" s="5"/>
-    </row>
-    <row r="14" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>29</v>
       </c>
@@ -1292,14 +2000,17 @@
         <v>11</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>104</v>
+        <v>99</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>109</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>90</v>
       </c>
       <c r="J14" s="5"/>
     </row>
-    <row r="15" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>29</v>
       </c>
@@ -1315,353 +2026,1985 @@
       <c r="E15" s="2" t="s">
         <v>100</v>
       </c>
+      <c r="F15" s="2" t="s">
+        <v>109</v>
+      </c>
       <c r="G15" s="2" t="s">
         <v>81</v>
       </c>
       <c r="J15" s="5"/>
     </row>
-    <row r="16" spans="1:10" s="12" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="9" t="s">
+    <row r="16" spans="1:12" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="C16" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D16" s="11" t="s">
+      <c r="D16" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="G16" s="11" t="s">
-        <v>111</v>
-      </c>
-      <c r="J16" s="9"/>
-    </row>
-    <row r="17" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
+      <c r="E16" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="G17" s="8"/>
+    </row>
+    <row r="18" spans="1:10" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="G18" s="8"/>
+    </row>
+    <row r="19" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B19" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C19" t="s">
         <v>40</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D19" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="G17" s="2" t="s">
+      <c r="E19" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="J17" s="5"/>
-    </row>
-    <row r="18" spans="1:10" s="12" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="s">
+    </row>
+    <row r="20" spans="1:10" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B20" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C20" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D20" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E18" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="G18" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="J18" s="9"/>
-    </row>
-    <row r="19" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="9" t="s">
+      <c r="E20" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="J20" s="6"/>
+    </row>
+    <row r="21" spans="1:10" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B21" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C19" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="E19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="J19" s="9"/>
-    </row>
-    <row r="20" spans="1:10" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
+      <c r="C21" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="G21" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="J21" s="6"/>
+    </row>
+    <row r="22" spans="1:10" s="9" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="G22" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="J22" s="6"/>
+    </row>
+    <row r="23" spans="1:10" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="G23" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="J23" s="6"/>
+    </row>
+    <row r="24" spans="1:10" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="J24" s="6"/>
+    </row>
+    <row r="25" spans="1:10" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B25" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C25" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D25" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E25" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="F20"/>
-      <c r="G20" s="4" t="s">
+      <c r="F25" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="G25" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="J20" s="6" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>33</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C21" t="s">
-        <v>30</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="J21" s="5"/>
-    </row>
-    <row r="22" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>33</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C22" t="s">
-        <v>41</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="J22" s="5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="60" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>33</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C23" t="s">
-        <v>31</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="J23" s="5"/>
-    </row>
-    <row r="24" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>33</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C24" t="s">
-        <v>28</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="J24" s="5"/>
-    </row>
-    <row r="25" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B25" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="J25" s="9"/>
     </row>
     <row r="26" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="C26" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>101</v>
+        <v>99</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>108</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="J26" s="5"/>
+        <v>77</v>
+      </c>
     </row>
     <row r="27" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="C27" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>101</v>
+        <v>99</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>108</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="J27" s="5"/>
     </row>
-    <row r="28" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C28" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>51</v>
+        <v>14</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>109</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>79</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="J28" s="5"/>
     </row>
     <row r="29" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>33</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C29" t="s">
+        <v>28</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="J29" s="5"/>
+    </row>
+    <row r="30" spans="1:10" s="9" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A30" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="G30" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="J30" s="6"/>
+    </row>
+    <row r="31" spans="1:10" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="G31" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="J31" s="6"/>
+    </row>
+    <row r="32" spans="1:10" s="9" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A32" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C32" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="G32" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="J32" s="6"/>
+    </row>
+    <row r="33" spans="1:10" s="9" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A33" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="F33" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="G33" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="J33" s="6"/>
+    </row>
+    <row r="34" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C34" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="F34" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="G34" s="8"/>
+      <c r="J34" s="6"/>
+    </row>
+    <row r="35" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>35</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C35" t="s">
+        <v>40</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="J35" s="5"/>
+    </row>
+    <row r="36" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C36" t="s">
+        <v>42</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="J36" s="5"/>
+    </row>
+    <row r="37" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>36</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B37" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C37" t="s">
+        <v>35</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>36</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C38" t="s">
         <v>41</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="D38" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E29" s="2" t="s">
+      <c r="E38" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="G29" s="2" t="s">
+      <c r="F38" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="G38" s="2" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row r="39" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>36</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B39" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C39" t="s">
         <v>30</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="D39" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="E39" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="G30" s="2" t="s">
+      <c r="F39" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="G39" s="2" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    <row r="40" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>36</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B40" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C40" t="s">
         <v>7</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="D40" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E31" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="G31" s="2" t="s">
+      <c r="E40" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="G40" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+    <row r="41" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>36</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B41" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C41" t="s">
         <v>40</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="D41" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="E41" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" s="9" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A42" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C42" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D42" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="E42" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="F42" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="G42" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="J42" s="6"/>
+    </row>
+    <row r="43" spans="1:10" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A43" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D43" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="E43" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="F43" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="G43" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="J43" s="6"/>
+    </row>
+    <row r="44" spans="1:10" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A44" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C44" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D44" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E44" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="F44" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="G44" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="J44" s="6"/>
+    </row>
+    <row r="45" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A45" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B45" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C45" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E45" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="F45" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G45" s="12" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A46" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B46" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C46" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D46" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="E46" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="F46" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G46" s="12" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A47" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B47" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C47" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D47" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E47" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="F47" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G47" s="12" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A48" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B48" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C48" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D48" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="E48" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="F48" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G48" s="12" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A49" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B49" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C49" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D49" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="E49" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="F49" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G49" s="12" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A50" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B50" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C50" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D50" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="E50" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="F50" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G50" s="12" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A51" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B51" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C51" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D51" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E51" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="F51" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="G51" s="12" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A52" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B52" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C52" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="D52" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E52" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="F52" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G52" s="12" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A53" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B53" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C53" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D53" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="E53" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="F53" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G53" s="12" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A54" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B54" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C54" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D54" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="E54" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="G32" s="2" t="s">
-        <v>98</v>
+      <c r="F54" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="G54" s="12" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A55" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B55" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C55" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D55" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="E55" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="F55" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="G55" s="12" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A56" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B56" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C56" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D56" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E56" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="F56" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="G56" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A57" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="B57" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C57" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D57" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E57" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="F57" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="G57" s="12" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A58" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="B58" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C58" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="D58" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="E58" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="F58" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="G58" s="12" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="A59" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="B59" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C59" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D59" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="E59" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="F59" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G59" s="12" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A60" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B60" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C60" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D60" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E60" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="F60" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G60" s="12" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A61" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B61" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C61" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D61" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E61" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="F61" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G61" s="12" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A62" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B62" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C62" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="D62" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E62" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="F62" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G62" s="12" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A63" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B63" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C63" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D63" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="E63" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="F63" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G63" s="12" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A64" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B64" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C64" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="D64" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="E64" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="F64" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G64" s="12" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A65" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B65" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C65" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D65" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E65" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="F65" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G65" s="12" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A66" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B66" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C66" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="D66" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E66" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="F66" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G66" s="12" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A67" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B67" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C67" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D67" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="E67" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="F67" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G67" s="12" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A68" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B68" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C68" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D68" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="E68" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="F68" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="G68" s="12" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A69" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B69" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C69" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D69" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E69" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="F69" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G69" s="12" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A70" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B70" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C70" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D70" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="E70" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="F70" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G70" s="12" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A71" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="B71" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C71" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D71" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E71" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="F71" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G71" s="12" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A72" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="B72" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C72" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="D72" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E72" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="F72" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G72" s="12" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A73" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="B73" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C73" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D73" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E73" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="F73" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="G73" s="12" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="A74" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="B74" s="12" t="s">
+        <v>157</v>
+      </c>
+      <c r="C74" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E74" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="F74" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G74" s="12" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A75" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="B75" s="12" t="s">
+        <v>157</v>
+      </c>
+      <c r="C75" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E75" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="F75" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G75" s="12" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A76" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="B76" s="12" t="s">
+        <v>157</v>
+      </c>
+      <c r="C76" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="D76" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E76" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="F76" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="G76" s="12" t="s">
+        <v>160</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H44" xr:uid="{A5B8861B-C05D-461E-8A99-E228C4472CAF}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H44">
+      <sortCondition ref="A1:A44"/>
+    </sortState>
+  </autoFilter>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B33F3714-16C6-461A-B996-FD2880AF594A}">
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr defaultColWidth="37.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="37.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="75.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
+        <v>166</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>188</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>193</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>196</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>197</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" s="12" t="s">
+        <v>201</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>202</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>203</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>204</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>207</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>208</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>212</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>217</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>222</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>227</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>229</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>232</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>233</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>234</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>235</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4526EDC6-B6FC-4365-B168-D06258ADE7C6}">
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr defaultColWidth="55.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="48.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="66.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
+        <v>240</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>241</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>242</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>245</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>246</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>249</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>250</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>252</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>253</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>254</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>256</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>257</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>261</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>265</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>266</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" s="12" t="s">
+        <v>268</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>269</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
+        <v>272</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>273</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>274</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
+        <v>276</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>277</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
+        <v>280</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>281</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>282</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
+        <v>284</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>286</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
+        <v>288</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>289</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>290</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="12" t="s">
+        <v>292</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>293</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>294</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
+        <v>296</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>297</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>298</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A17" s="12" t="s">
+        <v>300</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>301</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>302</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A18" s="12" t="s">
+        <v>304</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>305</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>306</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" s="12" t="s">
+        <v>308</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>309</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>310</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>311</v>
       </c>
     </row>
   </sheetData>

</xml_diff>